<commit_message>
Actualiza resultados ACV generados por los análisis
</commit_message>
<xml_diff>
--- a/data/resultados.xlsx
+++ b/data/resultados.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PGF\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TFM_Graficos_ACV\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860E09F8-6EAE-4E64-AF46-C1CDE0850FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C3B450-BD97-4A5C-AA3C-ADA93E400F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" tabRatio="841" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cerceda_1habeq_ReCiPe" sheetId="1" r:id="rId1"/>
@@ -697,13 +697,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15440,10 +15440,10 @@
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B38" s="53" t="s">
+      <c r="B38" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="C38" s="53"/>
+      <c r="C38" s="54"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B39" s="51">
@@ -15643,7 +15643,7 @@
       <c r="G13" s="52" t="s">
         <v>152</v>
       </c>
-      <c r="L13" s="54" t="s">
+      <c r="L13" s="55" t="s">
         <v>150</v>
       </c>
     </row>
@@ -15655,7 +15655,7 @@
         <v>24</v>
       </c>
       <c r="G14" s="52"/>
-      <c r="L14" s="54"/>
+      <c r="L14" s="55"/>
       <c r="M14" t="s">
         <v>151</v>
       </c>
@@ -16457,10 +16457,10 @@
       </c>
     </row>
     <row r="38" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="53" t="s">
+      <c r="B38" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="C38" s="53"/>
+      <c r="C38" s="54"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B39" s="51">
@@ -17343,10 +17343,10 @@
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B38" s="53" t="s">
+      <c r="B38" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="C38" s="53"/>
+      <c r="C38" s="54"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B39" s="51">
@@ -18228,10 +18228,10 @@
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B38" s="53" t="s">
+      <c r="B38" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="C38" s="53"/>
+      <c r="C38" s="54"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B39" s="51">
@@ -19356,12 +19356,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{270468F2-230B-1842-A630-B6F7B0660841}">
   <dimension ref="B4:F161"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="53" t="s">
+      <c r="B4" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="C4" s="53"/>
+      <c r="C4" s="54"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
@@ -19550,15 +19554,15 @@
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
-        <f>B6</f>
+        <f t="shared" ref="B16:C21" si="0">B6</f>
         <v>GWP</v>
       </c>
       <c r="C16">
-        <f>C6</f>
+        <f t="shared" si="0"/>
         <v>5.2493077970682748E-4</v>
       </c>
       <c r="D16">
-        <f>E6</f>
+        <f t="shared" ref="D16:D21" si="1">E6</f>
         <v>1.5616360356018316E-4</v>
       </c>
       <c r="E16" s="51"/>
@@ -19566,15 +19570,15 @@
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
-        <f>B7</f>
+        <f t="shared" si="0"/>
         <v>FEU</v>
       </c>
       <c r="C17">
-        <f>C7</f>
+        <f t="shared" si="0"/>
         <v>1.4255040368743772E-2</v>
       </c>
       <c r="D17">
-        <f>E7</f>
+        <f t="shared" si="1"/>
         <v>6.8202886524552648E-4</v>
       </c>
       <c r="E17" s="51"/>
@@ -19582,15 +19586,15 @@
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
-        <f>B8</f>
+        <f t="shared" si="0"/>
         <v>MEU</v>
       </c>
       <c r="C18">
-        <f>C8</f>
+        <f t="shared" si="0"/>
         <v>2.0665210911652958E-3</v>
       </c>
       <c r="D18">
-        <f>E8</f>
+        <f t="shared" si="1"/>
         <v>2.5776132834738158E-4</v>
       </c>
       <c r="E18" s="51"/>
@@ -19598,15 +19602,15 @@
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" t="str">
-        <f>B9</f>
+        <f t="shared" si="0"/>
         <v>TET</v>
       </c>
       <c r="C19">
-        <f>C9</f>
+        <f t="shared" si="0"/>
         <v>1.6047439313932057E-4</v>
       </c>
       <c r="D19">
-        <f>E9</f>
+        <f t="shared" si="1"/>
         <v>8.2777153720315594E-5</v>
       </c>
       <c r="E19" s="51"/>
@@ -19614,15 +19618,15 @@
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="str">
-        <f>B10</f>
+        <f t="shared" si="0"/>
         <v>FET</v>
       </c>
       <c r="C20">
-        <f>C10</f>
+        <f t="shared" si="0"/>
         <v>0.10095001411493257</v>
       </c>
       <c r="D20">
-        <f>E10</f>
+        <f t="shared" si="1"/>
         <v>1.0636856402092317E-3</v>
       </c>
       <c r="E20" s="51"/>
@@ -19630,15 +19634,15 @@
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="str">
-        <f>B11</f>
+        <f t="shared" si="0"/>
         <v>MET</v>
       </c>
       <c r="C21">
-        <f>C11</f>
+        <f t="shared" si="0"/>
         <v>7.4335648927955661E-2</v>
       </c>
       <c r="D21">
-        <f>E11</f>
+        <f t="shared" si="1"/>
         <v>8.0364597646734445E-4</v>
       </c>
       <c r="E21" s="51"/>
@@ -19662,11 +19666,11 @@
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C24" t="str">
-        <f t="shared" ref="C24:D24" si="0">C15</f>
+        <f t="shared" ref="C24:D24" si="2">C15</f>
         <v>Cerceda</v>
       </c>
       <c r="D24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Vedra</v>
       </c>
       <c r="E24" s="51"/>
@@ -19690,15 +19694,15 @@
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="str">
-        <f t="shared" ref="B26:B30" si="1">B17</f>
+        <f t="shared" ref="B26:C30" si="3">B17</f>
         <v>FEU</v>
       </c>
       <c r="C26">
-        <f t="shared" ref="C26:C30" si="2">C17/$C$20</f>
+        <f t="shared" ref="C26:C30" si="4">C17/$C$20</f>
         <v>0.14120889921336979</v>
       </c>
       <c r="D26">
-        <f t="shared" ref="D26:D30" si="3">D17/MAX($D$16:$D$21)</f>
+        <f t="shared" ref="D26:D30" si="5">D17/MAX($D$16:$D$21)</f>
         <v>0.6411940139676684</v>
       </c>
       <c r="E26" s="51"/>
@@ -19706,15 +19710,15 @@
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>MEU</v>
       </c>
       <c r="C27">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.0470736029937962E-2</v>
       </c>
       <c r="D27">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.24232848372069662</v>
       </c>
       <c r="E27" s="51"/>
@@ -19722,15 +19726,15 @@
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>TET</v>
       </c>
       <c r="C28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.5896421069997962E-3</v>
       </c>
       <c r="D28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>7.7821069112141969E-2</v>
       </c>
       <c r="E28" s="51"/>
@@ -19738,31 +19742,31 @@
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>FET</v>
       </c>
       <c r="C29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="D29">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="E29" s="51"/>
-      <c r="F29" s="55"/>
+      <c r="F29" s="53"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>MET</v>
       </c>
       <c r="C30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.73636095625825082</v>
       </c>
       <c r="D30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.75552959078141135</v>
       </c>
       <c r="E30" s="51"/>
@@ -19825,11 +19829,11 @@
         <v>137</v>
       </c>
       <c r="C37" s="51">
-        <f t="shared" ref="C37:D41" si="4">C26</f>
+        <f t="shared" ref="C37:D41" si="6">C26</f>
         <v>0.14120889921336979</v>
       </c>
       <c r="D37" s="51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.6411940139676684</v>
       </c>
       <c r="E37" s="51"/>
@@ -19840,11 +19844,11 @@
         <v>138</v>
       </c>
       <c r="C38" s="51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.0470736029937962E-2</v>
       </c>
       <c r="D38" s="51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.24232848372069662</v>
       </c>
       <c r="E38" s="51"/>
@@ -19855,11 +19859,11 @@
         <v>139</v>
       </c>
       <c r="C39" s="51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.5896421069997962E-3</v>
       </c>
       <c r="D39" s="51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.7821069112141969E-2</v>
       </c>
       <c r="E39" s="51"/>
@@ -19870,11 +19874,11 @@
         <v>140</v>
       </c>
       <c r="C40" s="51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="D40" s="51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="E40" s="51"/>
@@ -19885,11 +19889,11 @@
         <v>141</v>
       </c>
       <c r="C41" s="51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.73636095625825082</v>
       </c>
       <c r="D41" s="51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.75552959078141135</v>
       </c>
       <c r="E41" s="51"/>
@@ -19920,7 +19924,10 @@
       <c r="F45" s="51"/>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C46" s="51"/>
+      <c r="C46" s="51" t="str">
+        <f>C15</f>
+        <v>Cerceda</v>
+      </c>
       <c r="D46" s="51"/>
       <c r="E46" s="51"/>
       <c r="F46" s="51"/>
@@ -19944,7 +19951,10 @@
       <c r="F49" s="51"/>
     </row>
     <row r="50" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C50" s="51"/>
+      <c r="C50">
+        <f t="shared" ref="C50" si="7">C41</f>
+        <v>0.73636095625825082</v>
+      </c>
       <c r="D50" s="51"/>
       <c r="E50" s="51"/>
       <c r="F50" s="51"/>
@@ -20027,19 +20037,19 @@
         <v>136</v>
       </c>
       <c r="C155" s="8">
-        <f>-LOG(C6)</f>
+        <f t="shared" ref="C155:F160" si="8">-LOG(C6)</f>
         <v>3.2798979613051746</v>
       </c>
       <c r="D155" s="8">
-        <f>-LOG(D6)</f>
+        <f t="shared" si="8"/>
         <v>1.2044186125645167</v>
       </c>
       <c r="E155" s="8">
-        <f>-LOG(E6)</f>
+        <f t="shared" si="8"/>
         <v>3.8064201779801117</v>
       </c>
       <c r="F155" s="8">
-        <f>-LOG(F6)</f>
+        <f t="shared" si="8"/>
         <v>2.2863250840434528</v>
       </c>
     </row>
@@ -20048,19 +20058,19 @@
         <v>137</v>
       </c>
       <c r="C156" s="8">
-        <f>-LOG(C7)</f>
+        <f t="shared" si="8"/>
         <v>1.8460315484774368</v>
       </c>
       <c r="D156" s="8">
-        <f>-LOG(D7)</f>
+        <f t="shared" si="8"/>
         <v>-0.23419792030444103</v>
       </c>
       <c r="E156" s="8">
-        <f>-LOG(E7)</f>
+        <f t="shared" si="8"/>
         <v>3.1661972444761184</v>
       </c>
       <c r="F156" s="8">
-        <f>-LOG(F7)</f>
+        <f t="shared" si="8"/>
         <v>1.6418190808655977</v>
       </c>
     </row>
@@ -20069,19 +20079,19 @@
         <v>138</v>
       </c>
       <c r="C157" s="8">
-        <f>-LOG(C8)</f>
+        <f t="shared" si="8"/>
         <v>2.6847601578974136</v>
       </c>
       <c r="D157" s="8">
-        <f>-LOG(D8)</f>
+        <f t="shared" si="8"/>
         <v>0.60432627768030689</v>
       </c>
       <c r="E157" s="8">
-        <f>-LOG(E8)</f>
+        <f t="shared" si="8"/>
         <v>3.5887822388256509</v>
       </c>
       <c r="F157" s="8">
-        <f>-LOG(F8)</f>
+        <f t="shared" si="8"/>
         <v>2.0679374085207267</v>
       </c>
     </row>
@@ -20090,19 +20100,19 @@
         <v>139</v>
       </c>
       <c r="C158" s="8">
-        <f>-LOG(C9)</f>
+        <f t="shared" si="8"/>
         <v>3.7945942579975882</v>
       </c>
       <c r="D158" s="8">
-        <f>-LOG(D9)</f>
+        <f t="shared" si="8"/>
         <v>1.714191212545805</v>
       </c>
       <c r="E158" s="8">
-        <f>-LOG(E9)</f>
+        <f t="shared" si="8"/>
         <v>4.082089510827414</v>
       </c>
       <c r="F158" s="8">
-        <f>-LOG(F9)</f>
+        <f t="shared" si="8"/>
         <v>2.5612211937552498</v>
       </c>
     </row>
@@ -20111,19 +20121,19 @@
         <v>140</v>
       </c>
       <c r="C159" s="8">
-        <f>-LOG(C10)</f>
+        <f t="shared" si="8"/>
         <v>0.99589361599684612</v>
       </c>
       <c r="D159" s="8">
-        <f>-LOG(D10)</f>
+        <f t="shared" si="8"/>
         <v>-1.0844726510381169</v>
       </c>
       <c r="E159" s="8">
-        <f>-LOG(E10)</f>
+        <f t="shared" si="8"/>
         <v>2.9731867037088415</v>
       </c>
       <c r="F159" s="8">
-        <f>-LOG(F10)</f>
+        <f t="shared" si="8"/>
         <v>1.4526234575822972</v>
       </c>
     </row>
@@ -20132,19 +20142,19 @@
         <v>141</v>
       </c>
       <c r="C160" s="8">
-        <f>-LOG(C11)</f>
+        <f t="shared" si="8"/>
         <v>1.1288028629589002</v>
       </c>
       <c r="D160" s="8">
-        <f>-LOG(D11)</f>
+        <f t="shared" si="8"/>
         <v>-0.95156340325106903</v>
       </c>
       <c r="E160" s="8">
-        <f>-LOG(E11)</f>
+        <f t="shared" si="8"/>
         <v>3.0949352252900275</v>
       </c>
       <c r="F160" s="8">
-        <f>-LOG(F11)</f>
+        <f t="shared" si="8"/>
         <v>1.574383868255212</v>
       </c>
     </row>

</xml_diff>